<commit_message>
Support unattended monthly runs via Task Scheduler
Adds AUTO_NEXT_MONTH so the target year/month defaults to "next
month from today" instead of a hardcoded value, and persists each
run's seat1 cumulative counts/last-assigned dates to schedule_state.json
so fairness carries over automatically without copying numbers by
hand. Adds run_schedule_generator.bat as the Task Scheduler action,
and .gitignore for the generated state file (per-install runtime
data, not something to track in the repo).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01366ZVJkqrJ7xhi4niwtEQo
</commit_message>
<xml_diff>
--- a/2026년_10월_상담센터_근무표.xlsx
+++ b/2026년_10월_상담센터_근무표.xlsx
@@ -535,12 +535,12 @@
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>김윤정</t>
+          <t>김병성</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>이영숙</t>
+          <t>박민선</t>
         </is>
       </c>
     </row>
@@ -550,12 +550,12 @@
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>김병성</t>
+          <t>박민선</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>박민선</t>
+          <t>김민성</t>
         </is>
       </c>
     </row>
@@ -589,22 +589,22 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>김병성</t>
+          <t>김민성</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>박민선</t>
+          <t>박미나</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>김민성</t>
+          <t>이민정</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>박미나</t>
+          <t>김윤정</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -616,22 +616,22 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>김민성</t>
+          <t>박미나</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>박미나</t>
+          <t>이민정</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>이민정</t>
+          <t>김윤정</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>추의성</t>
+          <t>이영숙</t>
         </is>
       </c>
       <c r="E9" s="5" t="n"/>
@@ -666,41 +666,41 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>이민정</t>
+          <t>이영숙</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>김윤정</t>
+          <t>김병성</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>이영숙</t>
+          <t>박민선</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>김병성</t>
+          <t>김민성</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>박민선</t>
+          <t>박미나</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>추의성</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
           <t>김은숙</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>이영숙</t>
-        </is>
-      </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
           <t>추의성</t>
@@ -713,7 +713,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>김민성</t>
+          <t>김병성</t>
         </is>
       </c>
     </row>
@@ -747,54 +747,54 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>김민성</t>
+          <t>이민정</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>박미나</t>
+          <t>김윤정</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>이민정</t>
+          <t>이영숙</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>김윤정</t>
+          <t>김병성</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>이영숙</t>
+          <t>박민선</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>박미나</t>
+          <t>김윤정</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>이민정</t>
+          <t>이영숙</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>김윤정</t>
+          <t>추의성</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>추의성</t>
+          <t>김은숙</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>김은숙</t>
+          <t>김민성</t>
         </is>
       </c>
     </row>
@@ -828,54 +828,54 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>김병성</t>
+          <t>김민성</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>박민선</t>
+          <t>박미나</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>김민성</t>
+          <t>이민정</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>박미나</t>
+          <t>김윤정</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>이민정</t>
+          <t>이영숙</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>박민선</t>
+          <t>박미나</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
+          <t>이민정</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
           <t>추의성</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>김은숙</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>김병성</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>김윤정</t>
         </is>
       </c>
     </row>

</xml_diff>